<commit_message>
Changed manual xml parsing to use pandas read_xml() instead
</commit_message>
<xml_diff>
--- a/input_file/example_reference_substances.xlsx
+++ b/input_file/example_reference_substances.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Reference Substances" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="EDQM_check_2026_05_15" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="EDQM_check_2026_05_18" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Substances" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDQM_check_2026_05_15" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDQM_check_2026_05_18" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDQM_check_2026_05_21" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -54,6 +55,11 @@
       <color theme="1"/>
       <sz val="14"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -200,7 +206,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -227,12 +233,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -591,6 +598,24 @@
 </table>
 </file>
 
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EDQMCheck_20260521_191731" displayName="EDQMCheck_20260521_191731" ref="A1:I7" headerRowCount="1">
+  <autoFilter ref="A1:I7"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Substance Specific Code"/>
+    <tableColumn id="2" name="Substance Received Year"/>
+    <tableColumn id="3" name="Substance Received Index"/>
+    <tableColumn id="4" name="Substance"/>
+    <tableColumn id="5" name="Article No."/>
+    <tableColumn id="6" name="In Stock"/>
+    <tableColumn id="7" name="Category"/>
+    <tableColumn id="8" name="Supplier Batch No."/>
+    <tableColumn id="9" name="Current Batch"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -925,13 +950,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Internal Batch No.</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="12" t="n"/>
+      <c r="B1" s="12" t="n"/>
+      <c r="C1" s="13" t="n"/>
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
       <c r="F1" s="1" t="n"/>
@@ -2530,6 +2555,338 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Substance Specific Code</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Substance Received Year</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Substance Received Index</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Substance</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Article No.</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>Supplier Batch No.</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>Current Batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Citalopram for SST CRS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y0000855</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pharmacopeia CRS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Citalopram for SST CRS</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y0000855</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pharmacopeia CRS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Carbamazepine impurity A CRS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Y0000033</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pharmacopeia CRS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B5" t="n">
+        <v>26</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rosuvastatine Related Compound B</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1606037</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Pharmacopeia USP</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>F063S0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>R13880</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B6" t="n">
+        <v>26</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rosuvastatine Ketone</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1A00050</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pharmacopeia USP</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>R192P0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>R218Q0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B7" t="n">
+        <v>26</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simvastatine SST  CRS </t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Y0002069</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pharmacopeia CRS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2544,47 +2901,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Substance Specific Code</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Substance Received Year</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Substance Received Index</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>Substance</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Article No.</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>Supplier Batch No.</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="I1" s="14" t="inlineStr">
         <is>
           <t>Current Batch</t>
         </is>

</xml_diff>